<commit_message>
Updated BRA_grids_kan10 model - 2026-06-26 14:55
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA_grids_kan10/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_BRA_grids_kan10/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA_grids_kan10\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{55F49BCE-85B2-4BE4-A3E7-EA5F6EC121F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4523E12D-DE77-4ECB-8DDA-283574DD0BF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24833,7 +24833,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B49FE57-857B-4569-A8D4-E36A584D2EAA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{568E9C79-4F74-44F9-A2A7-32CE2E12CD30}">
   <dimension ref="B9:H248"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -29631,7 +29631,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2A0D142-63F9-422C-8855-19DC127E138A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{956F823F-C8F1-4ADC-AB05-785BDA0E67C5}">
   <dimension ref="B9:L248"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated BRA_grids_kan10 model - 2026-06-26 15:59
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA_grids_kan10/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_BRA_grids_kan10/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA_grids_kan10\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4523E12D-DE77-4ECB-8DDA-283574DD0BF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E0BA29CD-75BE-4D65-A216-A6FA6004A067}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24833,7 +24833,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{568E9C79-4F74-44F9-A2A7-32CE2E12CD30}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D28541D-30A7-4DF6-81B5-07515A068C0A}">
   <dimension ref="B9:H248"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -29631,7 +29631,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{956F823F-C8F1-4ADC-AB05-785BDA0E67C5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84EA8501-39EA-480F-A13E-D29DB3928357}">
   <dimension ref="B9:L248"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>